<commit_message>
Agrupa los hallazgos de previsión en uno solo
«Previsión inestable», «Previsión sin medición ni aprendizaje» y «Sin
previsión de demanda» pasan a ser HT-P2R-01 «Demanda sin previsión
fiable», curado por P2R-01. Se actualizan el maestro y las
intervenciones de Ondupet y Ondupack.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVYcGvnrywmVQkiA3sTncu
</commit_message>
<xml_diff>
--- a/maestros/Maestro_P2R_Hallazgos_Palancas.xlsx
+++ b/maestros/Maestro_P2R_Hallazgos_Palancas.xlsx
@@ -17,12 +17,12 @@
     <sheet name="Ondupet" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Detalle hallazgos'!$A$4:$J$38</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Detalle hallazgos'!$A$4:$J$39</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Detalle palancas'!$A$4:$K$28</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Hallazgos!$A$4:$M$16</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Hallazgos!$A$4:$M$15</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Otros procesos'!$A$4:$H$9</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Palancas!$A$4:$I$12</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Relación!$A$4:$E$17</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Relación!$A$4:$E$16</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="446">
   <si>
     <t xml:space="preserve">Maestro de hallazgos · Plan to Release (P2R) · nivel alto</t>
   </si>
@@ -90,10 +90,10 @@
     <t xml:space="preserve">Demanda y previsión</t>
   </si>
   <si>
-    <t xml:space="preserve">Previsión inestable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La previsión no se cierra ni se consensúa, cambia dentro del mes en curso y su horizonte no cubre las decisiones que alimenta.</t>
+    <t xml:space="preserve">Demanda sin previsión fiable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No hay previsión, o la que hay no se cierra, no se consensúa ni se mide: el plan trabaja con una demanda que cambia o que no se conoce, y la demanda perdida no se registra.</t>
   </si>
   <si>
     <t xml:space="preserve">Ineficiencia (coste)</t>
@@ -102,22 +102,13 @@
     <t xml:space="preserve">Circulante × CMPC</t>
   </si>
   <si>
-    <t xml:space="preserve">€ de previsión mensual cambiada tras el cierre o sin consensuar</t>
+    <t xml:space="preserve">€ de demanda mensual planificada sin previsión cerrada y consensuada</t>
   </si>
   <si>
     <t xml:space="preserve">PL01</t>
   </si>
   <si>
-    <t xml:space="preserve">H02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Previsión sin medición ni aprendizaje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se miden precisión ni sesgo, la demanda perdida no se registra y las desviaciones no llevan acción.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Familias fuera de umbral sin acción / mes</t>
+    <t xml:space="preserve">Agrupa «Previsión inestable», «Previsión sin medición ni aprendizaje» y «Sin previsión de demanda»: cada celda describe su caso.</t>
   </si>
   <si>
     <t xml:space="preserve">H03</t>
@@ -327,10 +318,7 @@
     <t xml:space="preserve">Gestión de la demanda</t>
   </si>
   <si>
-    <t xml:space="preserve">La previsión se cierra en fecha, se consensúa cada mes entre Comercial y Planificación, cubre el horizonte de las decisiones y se mide y corrige.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H01, H02</t>
+    <t xml:space="preserve">Hay previsión, al menos de la demanda repetitiva; se cierra en fecha, se consensúa cada mes entre Comercial y Planificación, cubre el horizonte de las decisiones y se mide y corrige.</t>
   </si>
   <si>
     <t xml:space="preserve">Precisión y sesgo por familia · cambios tras el cierre</t>
@@ -549,6 +537,18 @@
     <t xml:space="preserve">D-PL01</t>
   </si>
   <si>
+    <t xml:space="preserve">D-H45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No hay previsión: se planifica solo con la cartera, aunque haya clientes o referencias con consumo repetitivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€ de demanda repetitiva / mes sin previsión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso de Ondupack y de MGT.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D-H09</t>
   </si>
   <si>
@@ -903,6 +903,9 @@
     <t xml:space="preserve">Sí</t>
   </si>
   <si>
+    <t xml:space="preserve">D-H08, D-H45</t>
+  </si>
+  <si>
     <t xml:space="preserve">Precisión (1–WMAPE)</t>
   </si>
   <si>
@@ -1302,7 +1305,7 @@
     <t xml:space="preserve">Corrección manual de desviaciones de demanda</t>
   </si>
   <si>
-    <t xml:space="preserve">A confirmar: su detalle (antiguo H20) lo borraste; lo más cercano es H02.</t>
+    <t xml:space="preserve">A confirmar: su detalle (antiguo H20) lo borraste; lo más cercano es H01.</t>
   </si>
   <si>
     <t xml:space="preserve">Revisión de faltas manual</t>
@@ -1868,7 +1871,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1936,7 +1939,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
@@ -1968,59 +1971,63 @@
         <v>23</v>
       </c>
       <c r="K5" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A5)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A5)</f>
         <v>1</v>
       </c>
       <c r="L5" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A5)</f>
-        <v>3</v>
-      </c>
-      <c r="M5" s="5"/>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A5)</f>
+        <v>7</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K6" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A6)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A6)</f>
         <v>1</v>
       </c>
       <c r="L6" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A6)</f>
-        <v>3</v>
-      </c>
-      <c r="M6" s="5"/>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A6)</f>
+        <v>4</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>16</v>
@@ -2029,41 +2036,41 @@
         <v>2</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K7" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A7)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A7)</f>
         <v>1</v>
       </c>
       <c r="L7" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A7)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A7)</f>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>16</v>
@@ -2072,84 +2079,82 @@
         <v>2</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K8" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A8)</f>
-        <v>1</v>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A8)</f>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A8)</f>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A8)</f>
         <v>3</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="K9" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A9)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A9)</f>
+        <v>1</v>
       </c>
       <c r="L9" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A9)</f>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A9)</f>
         <v>3</v>
       </c>
-      <c r="M9" s="5" t="s">
-        <v>49</v>
-      </c>
+      <c r="M9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>16</v>
@@ -2158,80 +2163,80 @@
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K10" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A10)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A10)</f>
         <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A10)</f>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A10)</f>
         <v>3</v>
       </c>
       <c r="M10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="K11" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A11)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A11)</f>
         <v>1</v>
       </c>
       <c r="L11" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A11)</f>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A11)</f>
         <v>3</v>
       </c>
       <c r="M11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>16</v>
@@ -2240,121 +2245,123 @@
         <v>4</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K12" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A12)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A12)</f>
         <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A12)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A12)</f>
+        <v>2</v>
       </c>
       <c r="M12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="K13" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A13)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A13)</f>
         <v>1</v>
       </c>
       <c r="L13" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A13)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A13)</f>
+        <v>3</v>
       </c>
       <c r="M13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="K14" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A14)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A14)</f>
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A14)</f>
-        <v>3</v>
-      </c>
-      <c r="M14" s="5"/>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A14)</f>
+        <v>2</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>16</v>
@@ -2363,87 +2370,44 @@
         <v>6</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E15" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>82</v>
-      </c>
       <c r="K15" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A15)</f>
+        <f aca="false">COUNTIF(Relación!$C$5:$C$16,A15)</f>
         <v>1</v>
       </c>
       <c r="L15" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A15)</f>
+        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$39,A15)</f>
         <v>2</v>
       </c>
-      <c r="M15" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <f aca="false">COUNTIF(Relación!$C$5:$C$17,A16)</f>
-        <v>1</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <f aca="false">COUNTIF('Detalle hallazgos'!$G$5:$G$38,A16)</f>
-        <v>2</v>
-      </c>
-      <c r="M16" s="5"/>
+      <c r="M15" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M16"/>
-  <conditionalFormatting sqref="A5:M16">
+  <autoFilter ref="A4:M15"/>
+  <conditionalFormatting sqref="A5:M15">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>$G5="Oportunidad (ingreso expuesto)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K16">
+  <conditionalFormatting sqref="K5:K15">
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>$K5=0</formula>
     </cfRule>
@@ -2480,12 +2444,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2496,22 +2460,22 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>95</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>13</v>
@@ -2525,23 +2489,23 @@
         <v>16</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A5)</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A5)</f>
-        <v>2</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>100</v>
       </c>
       <c r="I5" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A5)</f>
@@ -2550,29 +2514,29 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F6" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A6)</f>
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A6)</f>
         <v>1</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I6" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A6)</f>
@@ -2581,29 +2545,29 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A7)</f>
+        <v>2</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A7)</f>
-        <v>2</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="I7" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A7)</f>
@@ -2612,29 +2576,29 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F8" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A8)</f>
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A8)</f>
         <v>1</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I8" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A8)</f>
@@ -2643,29 +2607,29 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A9)</f>
+        <v>2</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A9)</f>
-        <v>2</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A9)</f>
@@ -2674,29 +2638,29 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A10)</f>
+        <v>2</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A10)</f>
-        <v>2</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="I10" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A10)</f>
@@ -2705,29 +2669,29 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F11" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A11)</f>
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A11)</f>
         <v>1</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I11" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A11)</f>
@@ -2736,29 +2700,29 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <f aca="false">COUNTIF(Relación!$A$5:$A$16,A12)</f>
+        <v>2</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <f aca="false">COUNTIF(Relación!$A$5:$A$17,A12)</f>
-        <v>2</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="I12" s="4" t="n">
         <f aca="false">COUNTIF('Detalle palancas'!$I$5:$I$28,A12)</f>
@@ -2788,7 +2752,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2800,29 +2764,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2837,256 +2801,236 @@
         <v>15</v>
       </c>
       <c r="D5" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C5,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C5,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="E5" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C5,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C5,Hallazgos!$A$5:$A$15,0))</f>
         <v>Demanda y previsión</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A6,Palancas!$A$5:$A$12,0))</f>
-        <v>Gestión de la demanda</v>
+        <v>S&amp;OP y plan de capacidad</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C6,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión sin medición ni aprendizaje</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C6,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="E6" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C6,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Demanda y previsión</v>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C6,Hallazgos!$A$5:$A$15,0))</f>
+        <v>S&amp;OP y Plan Maestro</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A7,Palancas!$A$5:$A$12,0))</f>
-        <v>S&amp;OP y plan de capacidad</v>
+        <v>Política de inventario por segmento</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D7" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C7,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Demanda y capacidad sin equilibrar</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C7,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Stock sin política</v>
       </c>
       <c r="E7" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C7,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C7,Hallazgos!$A$5:$A$15,0))</f>
         <v>S&amp;OP y Plan Maestro</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A8,Palancas!$A$5:$A$12,0))</f>
         <v>Política de inventario por segmento</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D8" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C8,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Stock sin política</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C8,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Fecha al cliente no fiable</v>
       </c>
       <c r="E8" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C8,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C8,Hallazgos!$A$5:$A$15,0))</f>
         <v>S&amp;OP y Plan Maestro</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>40</v>
+        <v>106</v>
       </c>
       <c r="B9" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A9,Palancas!$A$5:$A$12,0))</f>
-        <v>Política de inventario por segmento</v>
+        <v>Promesa de fecha fiable</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D9" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C9,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C9,Hallazgos!$A$5:$A$15,0))</f>
         <v>Fecha al cliente no fiable</v>
       </c>
       <c r="E9" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C9,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C9,Hallazgos!$A$5:$A$15,0))</f>
         <v>S&amp;OP y Plan Maestro</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="B10" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A10,Palancas!$A$5:$A$12,0))</f>
-        <v>Promesa de fecha fiable</v>
+        <v>Planificación de materiales por excepción</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D10" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C10,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Fecha al cliente no fiable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C10,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Faltas tardías y gestionadas a mano</v>
       </c>
       <c r="E10" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C10,Hallazgos!$A$5:$A$16,0))</f>
-        <v>S&amp;OP y Plan Maestro</v>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C10,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Necesidades y Aprovisionamiento</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B11" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A11,Palancas!$A$5:$A$12,0))</f>
         <v>Planificación de materiales por excepción</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D11" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C11,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Faltas tardías y gestionadas a mano</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C11,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Necesidades poco fiables</v>
       </c>
       <c r="E11" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C11,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C11,Hallazgos!$A$5:$A$15,0))</f>
         <v>Necesidades y Aprovisionamiento</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B12" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A12,Palancas!$A$5:$A$12,0))</f>
-        <v>Planificación de materiales por excepción</v>
+        <v>Programación estable y optimizada</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C12,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Necesidades poco fiables</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C12,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Secuencia sin optimizar</v>
       </c>
       <c r="E12" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C12,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Necesidades y Aprovisionamiento</v>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C12,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Programación</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B13" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A13,Palancas!$A$5:$A$12,0))</f>
         <v>Programación estable y optimizada</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D13" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C13,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Secuencia sin optimizar</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C13,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Programa inestable</v>
       </c>
       <c r="E13" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C13,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C13,Hallazgos!$A$5:$A$15,0))</f>
         <v>Programación</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B14" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A14,Palancas!$A$5:$A$12,0))</f>
-        <v>Programación estable y optimizada</v>
+        <v>Liberación controlada</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D14" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C14,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Programa inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C14,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Liberación sin control</v>
       </c>
       <c r="E14" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C14,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Programación</v>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C14,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Liberación</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B15" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A15,Palancas!$A$5:$A$12,0))</f>
-        <v>Liberación controlada</v>
+        <v>Control del servicio y mejora continua</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D15" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C15,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Liberación sin control</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C15,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Servicio sin control</v>
       </c>
       <c r="E15" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C15,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Liberación</v>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C15,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Seguimiento y Control</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B16" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A16,Palancas!$A$5:$A$12,0))</f>
         <v>Control del servicio y mejora continua</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D16" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C16,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Servicio sin control</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(C16,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Ciclo sin aprendizaje</v>
       </c>
       <c r="E16" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C16,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$D$5:$D$15,MATCH(C16,Hallazgos!$A$5:$A$15,0))</f>
         <v>Seguimiento y Control</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="5" t="str">
-        <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(A17,Palancas!$A$5:$A$12,0))</f>
-        <v>Control del servicio y mejora continua</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(C17,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Ciclo sin aprendizaje</v>
-      </c>
-      <c r="E17" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$D$5:$D$16,MATCH(C17,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Seguimiento y Control</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:E17"/>
+  <autoFilter ref="A4:E16"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3103,7 +3047,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -3120,23 +3064,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>8</v>
@@ -3148,13 +3092,13 @@
         <v>10</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>14</v>
@@ -3162,13 +3106,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>20</v>
@@ -3177,29 +3121,29 @@
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G5,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G5,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="J5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>20</v>
@@ -3208,29 +3152,29 @@
         <v>21</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G6,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G6,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>20</v>
@@ -3239,31 +3183,31 @@
         <v>21</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H7" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G7,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión sin medición ni aprendizaje</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G7,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>20</v>
@@ -3272,29 +3216,29 @@
         <v>21</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H8" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G8,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión sin medición ni aprendizaje</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G8,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>20</v>
@@ -3303,157 +3247,157 @@
         <v>21</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H9" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G9,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión sin medición ni aprendizaje</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G9,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="J9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G10,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Previsión inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G10,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="H11" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G11,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Demanda y capacidad sin equilibrar</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G11,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H12" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G12,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G12,Hallazgos!$A$5:$A$15,0))</f>
         <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="J12" s="5"/>
+        <v>174</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="H13" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G13,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Stock sin política</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G13,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>183</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>20</v>
@@ -3462,453 +3406,455 @@
         <v>21</v>
       </c>
       <c r="F14" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G14,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Stock sin política</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G14,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="G15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G15,Hallazgos!$A$5:$A$15,0))</f>
         <v>Stock sin política</v>
       </c>
-      <c r="I14" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J14" s="5" t="s">
+      <c r="I15" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="5" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="B16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="5" t="s">
+      <c r="D16" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G16,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Fecha al cliente no fiable</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H15" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G15,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="E17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G17,Hallazgos!$A$5:$A$15,0))</f>
         <v>Fecha al cliente no fiable</v>
       </c>
-      <c r="I15" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="J15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="G16" s="4" t="s">
+      <c r="I17" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H16" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G16,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="E18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G18,Hallazgos!$A$5:$A$15,0))</f>
         <v>Fecha al cliente no fiable</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="J16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="H17" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G17,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Fecha al cliente no fiable</v>
-      </c>
-      <c r="I17" s="5" t="s">
+      <c r="I18" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="J17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G18,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Demanda y capacidad sin equilibrar</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>204</v>
-      </c>
+      <c r="J18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>32</v>
+        <v>201</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H19" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G19,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G19,Hallazgos!$A$5:$A$15,0))</f>
         <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="H20" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G20,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Necesidades poco fiables</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G20,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="J20" s="5"/>
+        <v>208</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H21" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G21,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Faltas tardías y gestionadas a mano</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G21,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Necesidades poco fiables</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="J21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>201</v>
+        <v>29</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="H22" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G22,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G22,Hallazgos!$A$5:$A$15,0))</f>
         <v>Faltas tardías y gestionadas a mano</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>54</v>
+        <v>201</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="H23" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G23,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G23,Hallazgos!$A$5:$A$15,0))</f>
         <v>Faltas tardías y gestionadas a mano</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="J23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="H24" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G24,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Necesidades poco fiables</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G24,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Faltas tardías y gestionadas a mano</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="J24" s="5"/>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H25" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G25,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G25,Hallazgos!$A$5:$A$15,0))</f>
         <v>Necesidades poco fiables</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="J25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="H26" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G26,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Stock sin política</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G26,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Necesidades poco fiables</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>109</v>
+        <v>232</v>
       </c>
       <c r="J26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="H27" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G27,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Secuencia sin optimizar</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G27,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Stock sin política</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>239</v>
+        <v>105</v>
       </c>
       <c r="J27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H28" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G28,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G28,Hallazgos!$A$5:$A$15,0))</f>
         <v>Secuencia sin optimizar</v>
       </c>
       <c r="I28" s="5" t="s">
@@ -3918,319 +3864,350 @@
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>70</v>
+        <v>242</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="H29" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G29,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Programa inestable</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G29,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Secuencia sin optimizar</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="J29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>201</v>
+        <v>29</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>248</v>
+        <v>67</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H30" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G30,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G30,Hallazgos!$A$5:$A$15,0))</f>
         <v>Programa inestable</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="J30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>32</v>
+        <v>201</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H31" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G31,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Secuencia sin optimizar</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G31,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Programa inestable</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="J31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>75</v>
+        <v>252</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="H32" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G32,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Liberación sin control</v>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G32,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Secuencia sin optimizar</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>128</v>
+        <v>239</v>
       </c>
       <c r="J32" s="5"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>257</v>
+        <v>72</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H33" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G33,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G33,Hallazgos!$A$5:$A$15,0))</f>
         <v>Liberación sin control</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H34" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G34,Hallazgos!$A$5:$A$16,0))</f>
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G34,Hallazgos!$A$5:$A$15,0))</f>
         <v>Liberación sin control</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="J34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H35" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G35,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Liberación sin control</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="J35" s="5"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C35" s="5" t="s">
+      <c r="B36" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F35" s="5" t="s">
+      <c r="D36" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="G35" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="H35" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G35,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="G36" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H36" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G36,Hallazgos!$A$5:$A$15,0))</f>
         <v>Servicio sin control</v>
       </c>
-      <c r="I35" s="5" t="s">
+      <c r="I36" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="J35" s="5" t="s">
+      <c r="J36" s="5" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="5" t="s">
+      <c r="B37" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F36" s="5" t="s">
+      <c r="D37" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="G36" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="H36" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G36,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="G37" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H37" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G37,Hallazgos!$A$5:$A$15,0))</f>
         <v>Servicio sin control</v>
       </c>
-      <c r="I36" s="5" t="s">
+      <c r="I37" s="5" t="s">
         <v>269</v>
-      </c>
-      <c r="J36" s="5"/>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H37" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G37,Hallazgos!$A$5:$A$16,0))</f>
-        <v>Ciclo sin aprendizaje</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>273</v>
       </c>
       <c r="J37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E38" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H38" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G38,Hallazgos!$A$5:$A$15,0))</f>
+        <v>Ciclo sin aprendizaje</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="J38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F39" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H38" s="5" t="str">
-        <f aca="false">INDEX(Hallazgos!$E$5:$E$16,MATCH(G38,Hallazgos!$A$5:$A$16,0))</f>
+      <c r="G39" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H39" s="5" t="str">
+        <f aca="false">INDEX(Hallazgos!$E$5:$E$15,MATCH(G39,Hallazgos!$A$5:$A$15,0))</f>
         <v>Ciclo sin aprendizaje</v>
       </c>
-      <c r="I38" s="5" t="s">
+      <c r="I39" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="J38" s="5"/>
+      <c r="J39" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J38"/>
-  <conditionalFormatting sqref="A5:J38">
+  <autoFilter ref="A4:J39"/>
+  <conditionalFormatting sqref="A5:J39">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>$D5="Oportunidad (ingreso expuesto)"</formula>
     </cfRule>
@@ -4278,7 +4255,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>279</v>
@@ -4296,13 +4273,13 @@
         <v>283</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>284</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>285</v>
@@ -4313,7 +4290,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>286</v>
@@ -4326,13 +4303,13 @@
         <v>288</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>167</v>
+        <v>289</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>23</v>
@@ -4345,26 +4322,26 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>23</v>
@@ -4377,26 +4354,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>23</v>
@@ -4409,26 +4386,26 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>23</v>
@@ -4441,26 +4418,26 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>23</v>
@@ -4476,26 +4453,26 @@
         <v>174</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J10" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I10,Palancas!$A$5:$A$12,0))</f>
@@ -4508,7 +4485,7 @@
         <v>179</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>287</v>
@@ -4521,13 +4498,13 @@
         <v>176</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J11" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I11,Palancas!$A$5:$A$12,0))</f>
@@ -4540,26 +4517,26 @@
         <v>245</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>243</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J12" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I12,Palancas!$A$5:$A$12,0))</f>
@@ -4569,31 +4546,31 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>287</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J13" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I13,Palancas!$A$5:$A$12,0))</f>
@@ -4603,29 +4580,29 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>191</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J14" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I14,Palancas!$A$5:$A$12,0))</f>
@@ -4638,26 +4615,26 @@
         <v>198</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>195</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J15" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I15,Palancas!$A$5:$A$12,0))</f>
@@ -4670,60 +4647,60 @@
         <v>203</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J16" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I16,Palancas!$A$5:$A$12,0))</f>
         <v>S&amp;OP y plan de capacidad</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>205</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J17" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I17,Palancas!$A$5:$A$12,0))</f>
@@ -4736,7 +4713,7 @@
         <v>221</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>287</v>
@@ -4749,13 +4726,13 @@
         <v>218</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J18" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I18,Palancas!$A$5:$A$12,0))</f>
@@ -4768,26 +4745,26 @@
         <v>213</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>210</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J19" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I19,Palancas!$A$5:$A$12,0))</f>
@@ -4800,26 +4777,26 @@
         <v>217</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J20" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I20,Palancas!$A$5:$A$12,0))</f>
@@ -4832,26 +4809,26 @@
         <v>228</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>225</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J21" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I21,Palancas!$A$5:$A$12,0))</f>
@@ -4864,26 +4841,26 @@
         <v>232</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>229</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J22" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I22,Palancas!$A$5:$A$12,0))</f>
@@ -4896,26 +4873,26 @@
         <v>239</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4" t="s">
         <v>288</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J23" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I23,Palancas!$A$5:$A$12,0))</f>
@@ -4928,14 +4905,14 @@
         <v>249</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>246</v>
@@ -4944,10 +4921,10 @@
         <v>248</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J24" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I24,Palancas!$A$5:$A$12,0))</f>
@@ -4957,29 +4934,29 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J25" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I25,Palancas!$A$5:$A$12,0))</f>
@@ -4992,26 +4969,26 @@
         <v>264</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="J26" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I26,Palancas!$A$5:$A$12,0))</f>
@@ -5024,26 +5001,26 @@
         <v>273</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
         <v>288</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="J27" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I27,Palancas!$A$5:$A$12,0))</f>
@@ -5053,36 +5030,36 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J28" s="5" t="str">
         <f aca="false">INDEX(Palancas!$C$5:$C$12,MATCH(I28,Palancas!$A$5:$A$12,0))</f>
         <v>Promesa de fecha fiable</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>
@@ -5117,12 +5094,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5130,10 +5107,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
@@ -5148,21 +5125,21 @@
         <v>10</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>20</v>
@@ -5171,24 +5148,24 @@
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>20</v>
@@ -5197,50 +5174,50 @@
         <v>201</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>20</v>
@@ -5249,24 +5226,24 @@
         <v>21</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>20</v>
@@ -5275,10 +5252,10 @@
         <v>21</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -5312,32 +5289,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,17 +5322,17 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C5,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C5,'Otros procesos'!$A$5:$A$9,0)))</f>
-        <v>Previsión inestable</v>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C5,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C5,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F5" s="5"/>
     </row>
@@ -5364,20 +5341,20 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D6" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C6,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C6,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C6,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C6,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>176</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,13 +5362,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D7" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C7,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C7,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C7,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C7,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Stock sin política</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -5404,20 +5381,20 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D8" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C8,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C8,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C8,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C8,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Demanda y capacidad sin equilibrar</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>199</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5425,20 +5402,20 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D9" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C9,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C9,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C9,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C9,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Fecha al cliente no fiable</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>195</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5446,18 +5423,18 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D10" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C10,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C10,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C10,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C10,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Cartera con errores (cantidades mayores que el pedido, fechas imposibles) y pedidos servidos sin saldar</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="5" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5465,18 +5442,18 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D11" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C11,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C11,'Otros procesos'!$A$5:$A$9,0)))</f>
-        <v>Previsión sin medición ni aprendizaje</v>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C11,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C11,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <v>Demanda sin previsión fiable</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="5" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5484,13 +5461,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D12" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C12,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C12,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C12,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C12,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Faltas tardías y gestionadas a mano</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -5503,13 +5480,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D13" s="5" t="str">
-        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$16,MATCH(C13,Hallazgos!$A$5:$A$16,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C13,'Otros procesos'!$A$5:$A$9,0)))</f>
+        <f aca="false">IFERROR(INDEX(Hallazgos!$E$5:$E$15,MATCH(C13,Hallazgos!$A$5:$A$15,0)),INDEX('Otros procesos'!$D$5:$D$9,MATCH(C13,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Secuencia sin optimizar</v>
       </c>
       <c r="E13" s="4" t="s">
@@ -5524,30 +5501,30 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>285</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>23</v>
@@ -5557,76 +5534,76 @@
         <v>Gestión de la demanda</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D18" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C18,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C18,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>S&amp;OP y plan de capacidad</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D19" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C19,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C19,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Política de inventario por segmento</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D20" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C20,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C20,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Promesa de fecha fiable</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D21" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C21,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C21,'Otros procesos'!$A$5:$A$9,0)))</f>
@@ -5637,39 +5614,39 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D22" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C22,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C22,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Planificación de materiales por excepción</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D23" s="5" t="str">
         <f aca="false">IFERROR(INDEX(Palancas!$C$5:$C$12,MATCH(C23,Palancas!$A$5:$A$12,0)),INDEX('Otros procesos'!$H$5:$H$9,MATCH(C23,'Otros procesos'!$A$5:$A$9,0)))</f>
         <v>Programación estable y optimizada</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F23" s="5"/>
     </row>

</xml_diff>